<commit_message>
Adjust max biomass to HT ratio value to 80
</commit_message>
<xml_diff>
--- a/preylib/Species.xlsx
+++ b/preylib/Species.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhydra-my.sharepoint.com/personal/ttinker_nhydra-eco_com/Documents/SOFA2/SOFA/preylib/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{A23D99A9-694F-4699-A28C-CA127BD4CD97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C82E814-EA2E-4C04-A05F-47BAD35F40DA}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{A23D99A9-694F-4699-A28C-CA127BD4CD97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD208E40-AA30-4594-9844-EF2AB218B8FD}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="1425" windowWidth="33870" windowHeight="19305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6705" yWindow="975" windowWidth="48345" windowHeight="18840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Species" sheetId="1" r:id="rId1"/>
@@ -1964,7 +1964,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567397</xdr:colOff>
-      <xdr:row>133</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2014,7 +2014,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>339298</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2064,7 +2064,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>534543</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2114,7 +2114,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>491490</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2164,7 +2164,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>231775</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2214,8 +2214,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>536518</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>371533</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2263,8 +2263,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>491490</xdr:colOff>
-      <xdr:row>93</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2313,7 +2313,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>459507</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2363,7 +2363,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>379690</xdr:colOff>
-      <xdr:row>112</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2413,7 +2413,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>536829</xdr:colOff>
-      <xdr:row>134</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2463,7 +2463,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>492252</xdr:colOff>
-      <xdr:row>93</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2513,7 +2513,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>650827</xdr:colOff>
-      <xdr:row>88</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2563,7 +2563,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>344562</xdr:colOff>
-      <xdr:row>121</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2613,7 +2613,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>492113</xdr:colOff>
-      <xdr:row>113</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2663,7 +2663,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>491490</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2713,7 +2713,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>377190</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2763,7 +2763,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>461772</xdr:colOff>
-      <xdr:row>115</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2813,7 +2813,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>565246</xdr:colOff>
-      <xdr:row>90</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2863,7 +2863,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>494172</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2913,7 +2913,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>491490</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2963,7 +2963,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>414500</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3013,7 +3013,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>413512</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3063,7 +3063,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>499524</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3113,7 +3113,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>536391</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3163,7 +3163,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>423849</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3213,8 +3213,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>418074</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>369628</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3263,7 +3263,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>492373</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3313,7 +3313,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>457972</xdr:colOff>
-      <xdr:row>55</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3363,7 +3363,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>416560</xdr:colOff>
-      <xdr:row>57</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3413,7 +3413,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>377190</xdr:colOff>
-      <xdr:row>110</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3463,7 +3463,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>414112</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3513,7 +3513,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>491490</xdr:colOff>
-      <xdr:row>87</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3563,7 +3563,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>565492</xdr:colOff>
-      <xdr:row>35</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3613,7 +3613,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1451072</xdr:colOff>
-      <xdr:row>35</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3663,7 +3663,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>489126</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3713,7 +3713,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>537083</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3763,7 +3763,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>613101</xdr:colOff>
-      <xdr:row>56</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3813,7 +3813,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>498815</xdr:colOff>
-      <xdr:row>89</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3863,7 +3863,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>377190</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3913,8 +3913,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1069854</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3963,8 +3963,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>719323</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4013,8 +4013,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4063,8 +4063,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>115</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4113,8 +4113,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4163,8 +4163,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>377190</xdr:colOff>
-      <xdr:row>119</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4213,7 +4213,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>460355</xdr:colOff>
-      <xdr:row>82</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4263,7 +4263,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>570016</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4313,7 +4313,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>538050</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4363,8 +4363,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>418737</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>1904</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373379</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4413,8 +4413,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4463,8 +4463,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>125</xdr:row>
-      <xdr:rowOff>1904</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>373379</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4513,8 +4513,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1099185</xdr:colOff>
-      <xdr:row>125</xdr:row>
-      <xdr:rowOff>1904</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>373379</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4564,7 +4564,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>493023</xdr:colOff>
       <xdr:row>103</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4613,8 +4613,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4663,8 +4663,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>568364</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4713,8 +4713,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>461016</xdr:colOff>
-      <xdr:row>138</xdr:row>
-      <xdr:rowOff>3869</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4813,8 +4813,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>496902</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4913,8 +4913,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>384808</xdr:colOff>
-      <xdr:row>95</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4963,8 +4963,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>530478</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5013,7 +5013,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>568223</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -5063,8 +5063,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>568223</xdr:colOff>
-      <xdr:row>108</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5113,8 +5113,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>377190</xdr:colOff>
-      <xdr:row>105</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5163,8 +5163,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>606505</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>380999</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>371474</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5213,8 +5213,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>683558</xdr:colOff>
-      <xdr:row>86</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5263,8 +5263,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567381</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5313,8 +5313,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>415796</xdr:colOff>
-      <xdr:row>133</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5363,8 +5363,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5413,8 +5413,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>460372</xdr:colOff>
-      <xdr:row>112</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5463,8 +5463,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>141</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5513,8 +5513,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>498152</xdr:colOff>
-      <xdr:row>132</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5563,8 +5563,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567354</xdr:colOff>
-      <xdr:row>102</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5613,8 +5613,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>529931</xdr:colOff>
-      <xdr:row>107</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5663,8 +5663,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567163</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5713,8 +5713,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>536374</xdr:colOff>
-      <xdr:row>120</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5763,8 +5763,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567690</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5813,8 +5813,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>117</xdr:row>
-      <xdr:rowOff>1906</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>373381</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5863,8 +5863,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>496371</xdr:colOff>
-      <xdr:row>130</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5913,8 +5913,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>758759</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5963,8 +5963,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497897</xdr:colOff>
-      <xdr:row>118</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6013,8 +6013,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>651972</xdr:colOff>
-      <xdr:row>131</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6063,8 +6063,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>453393</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>1904</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373379</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6113,8 +6113,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>529900</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6163,8 +6163,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>532055</xdr:colOff>
-      <xdr:row>142</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6213,8 +6213,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>383604</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6263,8 +6263,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567253</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6313,8 +6313,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567253</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6363,8 +6363,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>496904</xdr:colOff>
-      <xdr:row>143</xdr:row>
-      <xdr:rowOff>1906</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>373381</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6413,8 +6413,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6463,8 +6463,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>461190</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6513,7 +6513,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>491490</xdr:colOff>
-      <xdr:row>100</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6563,8 +6563,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>423255</xdr:colOff>
-      <xdr:row>69</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6613,8 +6613,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>574929</xdr:colOff>
-      <xdr:row>126</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6663,8 +6663,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>993175</xdr:colOff>
-      <xdr:row>129</xdr:row>
-      <xdr:rowOff>1906</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>373381</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6713,7 +6713,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>728472</xdr:colOff>
-      <xdr:row>123</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>377190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6762,8 +6762,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>992509</xdr:colOff>
-      <xdr:row>127</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>373379</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6811,8 +6811,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>454025</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>1906</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373381</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6861,8 +6861,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>270002</xdr:colOff>
-      <xdr:row>106</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6911,8 +6911,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>495911</xdr:colOff>
-      <xdr:row>100</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6961,8 +6961,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567690</xdr:colOff>
-      <xdr:row>110</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7011,8 +7011,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>121</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7061,8 +7061,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>572240</xdr:colOff>
-      <xdr:row>99</xdr:row>
-      <xdr:rowOff>1904</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>373379</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7111,8 +7111,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7161,8 +7161,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>568542</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7211,8 +7211,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>496545</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7261,8 +7261,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>565404</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7311,8 +7311,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>531749</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7361,8 +7361,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>567690</xdr:colOff>
-      <xdr:row>109</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7411,8 +7411,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>910460</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7461,8 +7461,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1595764</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7511,8 +7511,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>757079</xdr:colOff>
-      <xdr:row>73</xdr:row>
-      <xdr:rowOff>1906</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373381</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7560,8 +7560,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7610,7 +7610,7 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>497205</xdr:colOff>
-      <xdr:row>65</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -7660,8 +7660,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>495185</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7710,8 +7710,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>495173</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7760,8 +7760,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>575731</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>373380</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7810,8 +7810,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>606679</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7860,8 +7860,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>526669</xdr:colOff>
-      <xdr:row>92</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7910,8 +7910,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>492915</xdr:colOff>
-      <xdr:row>139</xdr:row>
-      <xdr:rowOff>3867</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375342</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7960,8 +7960,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>454025</xdr:colOff>
-      <xdr:row>140</xdr:row>
-      <xdr:rowOff>3868</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>375343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -8318,6 +8318,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R144"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8396,7 +8397,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -8440,7 +8441,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -8466,7 +8467,7 @@
         <v>79118</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -8498,7 +8499,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -8542,7 +8543,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -8586,7 +8587,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -8630,7 +8631,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -8659,7 +8660,7 @@
         <v>79452</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -8688,7 +8689,7 @@
         <v>81446</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10</v>
       </c>
@@ -8732,7 +8733,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>11</v>
       </c>
@@ -8776,7 +8777,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>12</v>
       </c>
@@ -8820,7 +8821,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>14</v>
       </c>
@@ -8864,7 +8865,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>15</v>
       </c>
@@ -8911,7 +8912,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>16</v>
       </c>
@@ -8943,7 +8944,7 @@
         <v>98670</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>17</v>
       </c>
@@ -8966,7 +8967,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>18</v>
       </c>
@@ -8995,7 +8996,7 @@
         <v>79451</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>19</v>
       </c>
@@ -9036,7 +9037,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>20</v>
       </c>
@@ -9080,7 +9081,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>21</v>
       </c>
@@ -9124,7 +9125,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>22</v>
       </c>
@@ -9165,7 +9166,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>24</v>
       </c>
@@ -9209,7 +9210,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>25</v>
       </c>
@@ -9253,7 +9254,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>26</v>
       </c>
@@ -9294,7 +9295,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>27</v>
       </c>
@@ -9323,7 +9324,7 @@
         <v>98435</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>28</v>
       </c>
@@ -9364,7 +9365,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>29</v>
       </c>
@@ -9405,7 +9406,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>30</v>
       </c>
@@ -9446,7 +9447,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>31</v>
       </c>
@@ -9490,7 +9491,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>32</v>
       </c>
@@ -9516,7 +9517,7 @@
         <v>157968</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>33</v>
       </c>
@@ -9557,7 +9558,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>34</v>
       </c>
@@ -9598,7 +9599,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>35</v>
       </c>
@@ -9639,7 +9640,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>36</v>
       </c>
@@ -9680,7 +9681,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>37</v>
       </c>
@@ -9703,7 +9704,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>38</v>
       </c>
@@ -9747,7 +9748,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>39</v>
       </c>
@@ -9791,7 +9792,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>40</v>
       </c>
@@ -9820,7 +9821,7 @@
         <v>81033</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>41</v>
       </c>
@@ -9867,7 +9868,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>42</v>
       </c>
@@ -9914,7 +9915,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>43</v>
       </c>
@@ -9958,7 +9959,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>44</v>
       </c>
@@ -9999,7 +10000,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>45</v>
       </c>
@@ -10031,7 +10032,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>46</v>
       </c>
@@ -10075,7 +10076,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>47</v>
       </c>
@@ -10116,7 +10117,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>48</v>
       </c>
@@ -10157,7 +10158,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>49</v>
       </c>
@@ -10195,7 +10196,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>50</v>
       </c>
@@ -10236,7 +10237,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>51</v>
       </c>
@@ -10280,7 +10281,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>52</v>
       </c>
@@ -10321,7 +10322,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>53</v>
       </c>
@@ -10362,7 +10363,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>54</v>
       </c>
@@ -10388,7 +10389,7 @@
         <v>64358</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>55</v>
       </c>
@@ -10432,7 +10433,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>56</v>
       </c>
@@ -10461,7 +10462,7 @@
         <v>79612</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>57</v>
       </c>
@@ -10487,7 +10488,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>58</v>
       </c>
@@ -10531,7 +10532,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>59</v>
       </c>
@@ -10575,7 +10576,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>60</v>
       </c>
@@ -10616,7 +10617,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>61</v>
       </c>
@@ -10657,7 +10658,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>62</v>
       </c>
@@ -10698,7 +10699,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>63</v>
       </c>
@@ -10743,7 +10744,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>64</v>
       </c>
@@ -10772,7 +10773,7 @@
         <v>81691</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>65</v>
       </c>
@@ -10817,7 +10818,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>66</v>
       </c>
@@ -10858,7 +10859,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>67</v>
       </c>
@@ -10893,7 +10894,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>68</v>
       </c>
@@ -10943,7 +10944,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>69</v>
       </c>
@@ -10984,7 +10985,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>70</v>
       </c>
@@ -11010,7 +11011,7 @@
         <v>156862</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>71</v>
       </c>
@@ -11045,7 +11046,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>72</v>
       </c>
@@ -11080,7 +11081,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>73</v>
       </c>
@@ -11124,7 +11125,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>74</v>
       </c>
@@ -11159,7 +11160,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>75</v>
       </c>
@@ -11194,7 +11195,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>76</v>
       </c>
@@ -11232,7 +11233,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>77</v>
       </c>
@@ -11258,7 +11259,7 @@
         <v>158140</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>78</v>
       </c>
@@ -11284,7 +11285,7 @@
         <v>158191</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>79</v>
       </c>
@@ -11328,7 +11329,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>80</v>
       </c>
@@ -11354,7 +11355,7 @@
         <v>166082</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>81</v>
       </c>
@@ -11398,7 +11399,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>82</v>
       </c>
@@ -11436,7 +11437,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>83</v>
       </c>
@@ -11503,7 +11504,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>85</v>
       </c>
@@ -11544,7 +11545,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>86</v>
       </c>
@@ -11567,7 +11568,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>87</v>
       </c>
@@ -11608,7 +11609,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>88</v>
       </c>
@@ -11652,7 +11653,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>89</v>
       </c>
@@ -11681,7 +11682,7 @@
         <v>97775</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>90</v>
       </c>
@@ -11722,7 +11723,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>92</v>
       </c>
@@ -11760,7 +11761,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>93</v>
       </c>
@@ -11804,7 +11805,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>94</v>
       </c>
@@ -11845,7 +11846,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>95</v>
       </c>
@@ -11883,7 +11884,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>96</v>
       </c>
@@ -11921,7 +11922,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>97</v>
       </c>
@@ -11962,7 +11963,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>98</v>
       </c>
@@ -12003,7 +12004,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="96" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>99</v>
       </c>
@@ -12047,7 +12048,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="97" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>100</v>
       </c>
@@ -12088,7 +12089,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>101</v>
       </c>
@@ -12126,7 +12127,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>102</v>
       </c>
@@ -12167,7 +12168,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>103</v>
       </c>
@@ -12205,7 +12206,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="101" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>104</v>
       </c>
@@ -12246,7 +12247,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="102" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>105</v>
       </c>
@@ -12287,7 +12288,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="103" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>106</v>
       </c>
@@ -12375,7 +12376,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>108</v>
       </c>
@@ -12416,7 +12417,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>109</v>
       </c>
@@ -12457,7 +12458,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>110</v>
       </c>
@@ -12504,7 +12505,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="108" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>111</v>
       </c>
@@ -12548,7 +12549,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>112</v>
       </c>
@@ -12589,7 +12590,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>113</v>
       </c>
@@ -12630,7 +12631,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>114</v>
       </c>
@@ -12674,7 +12675,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>115</v>
       </c>
@@ -12718,7 +12719,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>116</v>
       </c>
@@ -12759,7 +12760,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>117</v>
       </c>
@@ -12800,7 +12801,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>118</v>
       </c>
@@ -12847,7 +12848,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>119</v>
       </c>
@@ -12888,7 +12889,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="117" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>120</v>
       </c>
@@ -12932,7 +12933,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>121</v>
       </c>
@@ -12976,7 +12977,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>122</v>
       </c>
@@ -13020,7 +13021,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>123</v>
       </c>
@@ -13064,7 +13065,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>124</v>
       </c>
@@ -13105,7 +13106,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>125</v>
       </c>
@@ -13146,7 +13147,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>126</v>
       </c>
@@ -13181,7 +13182,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>127</v>
       </c>
@@ -13219,7 +13220,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="125" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>128</v>
       </c>
@@ -13260,7 +13261,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>129</v>
       </c>
@@ -13296,7 +13297,7 @@
       </c>
       <c r="R126" s="6"/>
     </row>
-    <row r="127" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>130</v>
       </c>
@@ -13335,7 +13336,7 @@
       </c>
       <c r="R127" s="6"/>
     </row>
-    <row r="128" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>131</v>
       </c>
@@ -13373,7 +13374,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>132</v>
       </c>
@@ -13412,7 +13413,7 @@
       </c>
       <c r="R129" s="6"/>
     </row>
-    <row r="130" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>133</v>
       </c>
@@ -13456,7 +13457,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>134</v>
       </c>
@@ -13500,7 +13501,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="132" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>135</v>
       </c>
@@ -13544,7 +13545,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>136</v>
       </c>
@@ -13588,7 +13589,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>137</v>
       </c>
@@ -13629,7 +13630,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>138</v>
       </c>
@@ -13667,7 +13668,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>139</v>
       </c>
@@ -13708,7 +13709,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>140</v>
       </c>
@@ -13749,7 +13750,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>141</v>
       </c>
@@ -13790,7 +13791,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>142</v>
       </c>
@@ -13831,7 +13832,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="140" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>143</v>
       </c>
@@ -13872,7 +13873,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="141" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>144</v>
       </c>
@@ -13916,7 +13917,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>145</v>
       </c>
@@ -13957,7 +13958,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>146</v>
       </c>
@@ -13995,7 +13996,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="144" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>147</v>
       </c>
@@ -14022,7 +14023,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P144" xr:uid="{133BA9D9-057F-482B-9A84-7C45123F4F37}"/>
+  <autoFilter ref="A1:P144" xr:uid="{133BA9D9-057F-482B-9A84-7C45123F4F37}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="Octopus"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R143">
     <sortCondition ref="A2:A143"/>
   </sortState>
@@ -14034,15 +14041,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007C85BEB69FC2D74FAF0CFFD217B4FC14" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710db677ec6c1f9e2ee7ec057b94e111">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6188df5f-cd89-4f8d-a557-25c3c9ac281d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b477d7946c345dc1bd1ea843bd6a9161" ns2:_="">
     <xsd:import namespace="6188df5f-cd89-4f8d-a557-25c3c9ac281d"/>
@@ -14174,6 +14172,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -14181,14 +14188,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{701BD999-73B0-4962-BCE6-126EFE86DF99}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC9E02A9-0E2F-49B5-9C17-D38DD2951BA2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14202,6 +14201,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{701BD999-73B0-4962-BCE6-126EFE86DF99}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>